<commit_message>
feat: add new LFP, NMC, and SC configuration experiment files
</commit_message>
<xml_diff>
--- a/MultiCellBMSConfig/LFP/Experiment_1_LFP_Configuration.xlsx
+++ b/MultiCellBMSConfig/LFP/Experiment_1_LFP_Configuration.xlsx
@@ -572,7 +572,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Variable-Length CAN Mode: Set parser_type = 'waveshare_can' or 'variable_length' (Header 0xAA, DLC, CAN ID, payload, footer 0x55).</t>
+          <t xml:space="preserve">   - Variable-Length CAN Mode: Set parser_type = 'waveshare_can_variable_length' (Variable-Length CAN) (Header 0xAA, DLC, CAN ID, payload, footer 0x55).</t>
         </is>
       </c>
     </row>
@@ -891,12 +891,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>waveshare_can_20_bytes</t>
+          <t>waveshare_can_variable_length</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AA 55</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -938,7 +938,11 @@
           <t>header_to_payload</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>none</t>
@@ -962,7 +966,7 @@
   </sheetData>
   <dataValidations count="13">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"framed,waveshare_can,waveshare_can_20_bytes"</formula1>
+      <formula1>"framed,waveshare_can_variable_length,waveshare_can_20_bytes"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,4"</formula1>
@@ -1497,7 +1501,6 @@
       <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>little</t>
@@ -1558,7 +1561,6 @@
       <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>little</t>
@@ -2186,7 +2188,6 @@
       <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>little</t>
@@ -2247,7 +2248,6 @@
       <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>little</t>
@@ -2308,7 +2308,6 @@
       <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>little</t>
@@ -2794,7 +2793,6 @@
           <t>V</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="b">
         <v>1</v>
       </c>
@@ -2815,7 +2813,6 @@
           <t>V</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="b">
         <v>1</v>
       </c>
@@ -2836,7 +2833,6 @@
           <t>°C</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="b">
         <v>1</v>
       </c>
@@ -2857,7 +2853,6 @@
           <t>°C</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="b">
         <v>1</v>
       </c>

</xml_diff>